<commit_message>
Update volume_calculator.xlsx template with latest changes
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/volume_calculator.xlsx
+++ b/volume_calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\darta\Desktop\Bens\Work\Python\JUNC\git\JUNC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\PycharmProjects\ClaudeCode\JUNC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E367142D-CC8B-447D-83EE-AAEC5F7CD822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EBE88C-A7CE-4E7A-B439-A1CA8FC58BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="מחשבון נפח קובע" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="70">
   <si>
     <t>שמות הרחובות</t>
   </si>
@@ -492,24 +492,12 @@
   <si>
     <t>ערכי קיבולת לצומת לפי מספר פאזות</t>
   </si>
-  <si>
-    <t>קו סגול</t>
-  </si>
-  <si>
-    <t>לוי אשכול</t>
-  </si>
-  <si>
-    <t>יהודה הלוי</t>
-  </si>
-  <si>
-    <t>מיכאל וולך</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1688,6 +1676,54 @@
     <xf numFmtId="0" fontId="19" fillId="15" borderId="47" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="2"/>
     </xf>
@@ -1793,69 +1829,21 @@
     <xf numFmtId="0" fontId="14" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="1" fontId="10" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
-    <cellStyle name="20% - Accent1" xfId="4" builtinId="30"/>
-    <cellStyle name="Calculation" xfId="2" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="5" builtinId="23"/>
-    <cellStyle name="Input" xfId="1" builtinId="20"/>
+    <cellStyle name="20% - הדגשה1" xfId="4" builtinId="30"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Output" xfId="3" builtinId="21"/>
+    <cellStyle name="חישוב" xfId="2" builtinId="22"/>
+    <cellStyle name="פלט" xfId="3" builtinId="21"/>
+    <cellStyle name="קלט" xfId="1" builtinId="20"/>
+    <cellStyle name="תא מסומן" xfId="5" builtinId="23"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C6500"/>
@@ -1863,6 +1851,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1883,26 +1881,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2173,51 +2151,51 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AP46"/>
-  <sheetFormatPr defaultColWidth="11.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="13.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="4.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="11.88671875" style="8"/>
-    <col min="36" max="36" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="13.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="4.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="11.85546875" style="8"/>
+    <col min="36" max="36" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="4.7109375" style="8" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="5" style="8" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="5.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="11.88671875" style="8"/>
-    <col min="41" max="41" width="6.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="23.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="43" max="16384" width="11.88671875" style="8"/>
+    <col min="39" max="39" width="5.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.85546875" style="8"/>
+    <col min="41" max="41" width="6.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="23.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="43" max="16384" width="11.85546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="7"/>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -2244,49 +2222,49 @@
       <c r="X1" s="7"/>
       <c r="Y1" s="7"/>
     </row>
-    <row r="2" spans="1:42" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:42" ht="16.5">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
-      <c r="C2" s="119" t="str">
+      <c r="C2" s="135" t="str">
         <f>IF(ISBLANK(V4),"צפון","צפון   -   "&amp;V4)</f>
-        <v>צפון   -   לוי אשכול</v>
-      </c>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="122" t="str">
+        <v>צפון</v>
+      </c>
+      <c r="D2" s="136"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138" t="str">
         <f>IF(ISBLANK(W4),"דרום","דרום   -   "&amp;W4)</f>
-        <v>דרום   -   לוי אשכול</v>
-      </c>
-      <c r="H2" s="123"/>
-      <c r="I2" s="123"/>
-      <c r="J2" s="124"/>
-      <c r="K2" s="125" t="str">
+        <v>דרום</v>
+      </c>
+      <c r="H2" s="139"/>
+      <c r="I2" s="139"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="141" t="str">
         <f>IF(ISBLANK(X4),"מזרח","מזרח   -   "&amp;X4)</f>
-        <v>מזרח   -   יהודה הלוי</v>
-      </c>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="127"/>
-      <c r="O2" s="128" t="str">
+        <v>מזרח</v>
+      </c>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="143"/>
+      <c r="O2" s="144" t="str">
         <f>IF(ISBLANK(Y4),"מערב","מערב   -   "&amp;Y4)</f>
-        <v>מערב   -   מיכאל וולך</v>
-      </c>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="130"/>
+        <v>מערב</v>
+      </c>
+      <c r="P2" s="145"/>
+      <c r="Q2" s="145"/>
+      <c r="R2" s="146"/>
       <c r="S2" s="7"/>
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
-      <c r="V2" s="131" t="s">
-        <v>0</v>
-      </c>
-      <c r="W2" s="132"/>
-      <c r="X2" s="132"/>
-      <c r="Y2" s="133"/>
+      <c r="V2" s="147" t="s">
+        <v>0</v>
+      </c>
+      <c r="W2" s="148"/>
+      <c r="X2" s="148"/>
+      <c r="Y2" s="149"/>
       <c r="AN2" s="9"/>
     </row>
-    <row r="3" spans="1:42" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:42" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="10" t="s">
@@ -2356,74 +2334,34 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:42" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:42" ht="15.75" customHeight="1" thickBot="1">
       <c r="A4" s="7"/>
       <c r="B4" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="27">
-        <v>927</v>
-      </c>
-      <c r="D4" s="28">
-        <v>107</v>
-      </c>
-      <c r="E4" s="28">
-        <v>760</v>
-      </c>
-      <c r="F4" s="29">
-        <v>60</v>
-      </c>
-      <c r="G4" s="27">
-        <v>1211</v>
-      </c>
-      <c r="H4" s="28">
-        <v>73</v>
-      </c>
-      <c r="I4" s="28">
-        <v>333</v>
-      </c>
-      <c r="J4" s="29">
-        <v>193</v>
-      </c>
-      <c r="K4" s="27">
-        <v>750</v>
-      </c>
-      <c r="L4" s="28">
-        <v>500</v>
-      </c>
-      <c r="M4" s="28">
-        <v>368</v>
-      </c>
-      <c r="N4" s="29">
-        <v>180</v>
-      </c>
-      <c r="O4" s="27">
-        <v>453</v>
-      </c>
-      <c r="P4" s="28">
-        <v>177</v>
-      </c>
-      <c r="Q4" s="28">
-        <v>177</v>
-      </c>
-      <c r="R4" s="29">
-        <v>99</v>
-      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="29"/>
       <c r="S4" s="7"/>
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
-      <c r="V4" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="W4" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="X4" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>73</v>
-      </c>
+      <c r="V4" s="30"/>
+      <c r="W4" s="31"/>
+      <c r="X4" s="31"/>
+      <c r="Y4" s="32"/>
       <c r="AO4" s="33" t="b">
         <f>AND(D4&gt;0,C8+D8+H8+I8&lt;1)</f>
         <v>0</v>
@@ -2432,59 +2370,27 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:42" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:42" ht="15.75" customHeight="1" thickBot="1">
       <c r="A5" s="7"/>
       <c r="B5" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="35">
-        <v>980</v>
-      </c>
-      <c r="D5" s="36">
-        <v>59</v>
-      </c>
-      <c r="E5" s="36">
-        <v>735</v>
-      </c>
-      <c r="F5" s="37">
-        <v>186</v>
-      </c>
-      <c r="G5" s="35">
-        <v>1100</v>
-      </c>
-      <c r="H5" s="36">
-        <v>115</v>
-      </c>
-      <c r="I5" s="36">
-        <v>825</v>
-      </c>
-      <c r="J5" s="37">
-        <v>160</v>
-      </c>
-      <c r="K5" s="35">
-        <v>433</v>
-      </c>
-      <c r="L5" s="36">
-        <v>113</v>
-      </c>
-      <c r="M5" s="36">
-        <v>186</v>
-      </c>
-      <c r="N5" s="37">
-        <v>134</v>
-      </c>
-      <c r="O5" s="35">
-        <v>763</v>
-      </c>
-      <c r="P5" s="36">
-        <v>287</v>
-      </c>
-      <c r="Q5" s="36">
-        <v>234</v>
-      </c>
-      <c r="R5" s="37">
-        <v>242</v>
-      </c>
+      <c r="C5" s="35"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="35"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="36"/>
+      <c r="R5" s="37"/>
       <c r="S5" s="7"/>
       <c r="T5" s="7"/>
       <c r="U5" s="7"/>
@@ -2495,7 +2401,7 @@
       <c r="AO5" s="33"/>
       <c r="AP5" s="33"/>
     </row>
-    <row r="6" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:42" ht="15.75" thickBot="1">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -2529,7 +2435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:42" ht="16.5" thickBot="1">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="38" t="s">
@@ -2626,16 +2532,16 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:42" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:42" ht="15.75" customHeight="1" thickBot="1">
       <c r="A8" s="7"/>
       <c r="B8" s="46" t="s">
         <v>22</v>
       </c>
       <c r="C8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="47">
         <v>0</v>
@@ -2644,7 +2550,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="47">
         <v>0</v>
@@ -2654,19 +2560,19 @@
       </c>
       <c r="J8" s="49"/>
       <c r="K8" s="47">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P8" s="47">
         <v>0</v>
@@ -2676,7 +2582,7 @@
       </c>
       <c r="R8" s="49"/>
       <c r="S8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8" s="47">
         <v>0</v>
@@ -2685,10 +2591,10 @@
         <v>0</v>
       </c>
       <c r="V8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X8" s="47">
         <v>0</v>
@@ -2698,19 +2604,19 @@
       </c>
       <c r="Z8" s="49"/>
       <c r="AA8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="47">
         <v>0</v>
       </c>
       <c r="AD8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="47">
         <v>0</v>
@@ -2726,7 +2632,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:42" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:42" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="7"/>
       <c r="B9" s="50" t="s">
         <v>24</v>
@@ -2735,7 +2641,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="47">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="47">
         <v>0</v>
@@ -2754,16 +2660,16 @@
       </c>
       <c r="J9" s="49"/>
       <c r="K9" s="47">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L9" s="47">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M9" s="47">
         <v>0</v>
       </c>
       <c r="N9" s="47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O9" s="47">
         <v>0</v>
@@ -2776,7 +2682,7 @@
       </c>
       <c r="R9" s="49"/>
       <c r="S9" s="47">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="T9" s="47">
         <v>0</v>
@@ -2785,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="V9" s="47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W9" s="47">
         <v>0</v>
@@ -2801,13 +2707,13 @@
         <v>0</v>
       </c>
       <c r="AB9" s="47">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="47">
         <v>0</v>
       </c>
       <c r="AD9" s="47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="47">
         <v>0</v>
@@ -2821,7 +2727,7 @@
       <c r="AO9" s="33"/>
       <c r="AP9" s="33"/>
     </row>
-    <row r="10" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A10" s="7"/>
       <c r="B10" s="7" t="s">
         <v>25</v>
@@ -2896,7 +2802,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A11" s="7"/>
       <c r="B11" s="7" t="s">
         <v>28</v>
@@ -2982,7 +2888,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A12" s="7"/>
       <c r="B12" s="7" t="s">
         <v>30</v>
@@ -3049,19 +2955,19 @@
       </c>
       <c r="AJ12" s="8">
         <f>IF(C8&gt;9,0,D4)</f>
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="AK12" s="8">
         <f>IF(K8&gt;9,0,H4)</f>
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="AL12" s="8">
         <f>IF(S8&gt;9,0,L4)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="AM12" s="8">
         <f>IF(AA8&gt;9,0,P4)</f>
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="AO12" s="33" t="b">
         <f>AND(L4&gt;0,S8+T8+X8+Y8&lt;1)</f>
@@ -3071,7 +2977,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="7" t="s">
         <v>1</v>
@@ -3198,7 +3104,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="57"/>
@@ -3234,15 +3140,15 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="7">
         <f>C15+K15+S15+AA15</f>
-        <v>1070210.1072277033</v>
+        <v>0</v>
       </c>
       <c r="C15" s="57">
         <f>C13^2*C8+D13^2*D8+E13^2*E8+F13^2*F8+G13^2*G8+H13^2*H8+I13^2*I8</f>
-        <v>14999.999999999998</v>
+        <v>0</v>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
@@ -3253,7 +3159,7 @@
       <c r="J15" s="7"/>
       <c r="K15" s="57">
         <f>K13^2*K8+L13^2*L8+M13^2*M8+N13^2*N8+O13^2*O8+P13^2*P8+Q13^2*Q8</f>
-        <v>612710.10722770332</v>
+        <v>0</v>
       </c>
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
@@ -3264,7 +3170,7 @@
       <c r="R15" s="7"/>
       <c r="S15" s="57">
         <f>S13^2*S8+T13^2*T8+U13^2*U8+V13^2*V8+W13^2*W8+X13^2*X8+Y13^2*Y8</f>
-        <v>102500</v>
+        <v>0</v>
       </c>
       <c r="T15" s="7"/>
       <c r="U15" s="7"/>
@@ -3274,7 +3180,7 @@
       <c r="Y15" s="58"/>
       <c r="AA15" s="59">
         <f>AA13^2*AA8+AB13^2*AB8+AC13^2*AC8+AD13^2*AD8+AE13^2*AE8+AF13^2*AF8+AG13^2*AG8</f>
-        <v>340000</v>
+        <v>0</v>
       </c>
       <c r="AG15" s="60"/>
       <c r="AO15" s="33" t="b">
@@ -3285,7 +3191,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="57"/>
@@ -3321,18 +3227,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A17" s="61"/>
       <c r="B17" s="61" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="62">
         <f t="shared" ref="C17:I17" si="4">IF(C8&gt;0,C13,0)</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D17" s="63">
         <f t="shared" si="4"/>
-        <v>49.999999999999986</v>
+        <v>0</v>
       </c>
       <c r="E17" s="63">
         <f t="shared" si="4"/>
@@ -3344,7 +3250,7 @@
       </c>
       <c r="G17" s="63">
         <f t="shared" si="4"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H17" s="63">
         <f t="shared" si="4"/>
@@ -3357,23 +3263,23 @@
       <c r="J17" s="7"/>
       <c r="K17" s="62">
         <f t="shared" ref="K17:Q17" si="5">IF(K8&gt;0,K13,0)</f>
-        <v>33.333333333333343</v>
+        <v>0</v>
       </c>
       <c r="L17" s="63">
         <f t="shared" si="5"/>
-        <v>761.45000638761621</v>
+        <v>0</v>
       </c>
       <c r="M17" s="63">
         <f t="shared" si="5"/>
-        <v>49.999950000000013</v>
+        <v>0</v>
       </c>
       <c r="N17" s="63">
         <f t="shared" si="5"/>
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="O17" s="63">
         <f t="shared" si="5"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P17" s="63">
         <f t="shared" si="5"/>
@@ -3386,7 +3292,7 @@
       <c r="R17" s="7"/>
       <c r="S17" s="62">
         <f t="shared" ref="S17:Y17" si="6">IF(S8&gt;0,S13,0)</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="T17" s="63">
         <f t="shared" si="6"/>
@@ -3398,11 +3304,11 @@
       </c>
       <c r="V17" s="63">
         <f t="shared" si="6"/>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="W17" s="63">
         <f t="shared" si="6"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="X17" s="63">
         <f t="shared" si="6"/>
@@ -3419,7 +3325,7 @@
       </c>
       <c r="AB17" s="66">
         <f t="shared" si="7"/>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="AC17" s="66">
         <f t="shared" si="7"/>
@@ -3427,7 +3333,7 @@
       </c>
       <c r="AD17" s="66">
         <f t="shared" si="7"/>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="AE17" s="66">
         <f t="shared" si="7"/>
@@ -3450,7 +3356,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A18" s="61" t="s">
         <v>38</v>
       </c>
@@ -3460,7 +3366,7 @@
       <c r="E18" s="61"/>
       <c r="F18" s="61">
         <f>MAX(C17:I17)</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G18" s="61"/>
       <c r="H18" s="61"/>
@@ -3471,7 +3377,7 @@
       <c r="M18" s="61"/>
       <c r="N18" s="61">
         <f>MAX(K17:Q17)</f>
-        <v>761.45000638761621</v>
+        <v>0</v>
       </c>
       <c r="O18" s="61"/>
       <c r="P18" s="61"/>
@@ -3482,7 +3388,7 @@
       <c r="U18" s="61"/>
       <c r="V18" s="61">
         <f>MAX(S17:Y17)</f>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="W18" s="61"/>
       <c r="X18" s="61"/>
@@ -3491,7 +3397,7 @@
       <c r="AA18" s="72"/>
       <c r="AD18" s="68">
         <f>MAX(AA17:AG17)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="AG18" s="73"/>
       <c r="AH18" s="8"/>
@@ -3502,7 +3408,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:42" s="68" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A19" s="61" t="s">
         <v>40</v>
       </c>
@@ -3510,12 +3416,12 @@
       <c r="C19" s="70"/>
       <c r="D19" s="61">
         <f>IF(F$8+H$8+I$8+N$8+P$8+Q$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E19" s="61"/>
       <c r="F19" s="61">
         <f>MAX(C17:F17,H17:I17,K17:N17,P17:Q17)</f>
-        <v>761.45000638761621</v>
+        <v>0</v>
       </c>
       <c r="G19" s="61"/>
       <c r="H19" s="61"/>
@@ -3526,7 +3432,7 @@
       <c r="M19" s="61"/>
       <c r="N19" s="61">
         <f>MAX(G17,O17)+D19</f>
-        <v>10100</v>
+        <v>0</v>
       </c>
       <c r="O19" s="61"/>
       <c r="P19" s="61"/>
@@ -3535,12 +3441,12 @@
       <c r="S19" s="70"/>
       <c r="T19" s="61">
         <f>IF(V$8+X$8+Y$8+AD$8+AF$8+AG$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="U19" s="61"/>
       <c r="V19" s="61">
         <f>MAX(S17:V17,X17:Y17,AA17:AD17,AF17:AG17)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="W19" s="61"/>
       <c r="X19" s="61"/>
@@ -3549,7 +3455,7 @@
       <c r="AA19" s="72"/>
       <c r="AD19" s="68">
         <f>MAX(W17,AE17)+T19</f>
-        <v>10050</v>
+        <v>0</v>
       </c>
       <c r="AG19" s="73"/>
       <c r="AH19" s="8"/>
@@ -3558,20 +3464,20 @@
         <v>תקין</v>
       </c>
     </row>
-    <row r="20" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="134" t="s">
+    <row r="20" spans="1:42" s="68" customFormat="1" hidden="1">
+      <c r="A20" s="99" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="134"/>
+      <c r="B20" s="99"/>
       <c r="C20" s="70"/>
       <c r="D20" s="61">
         <f>IF(F$8+H$8+I$8+G$8+N$8+P$8+Q$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E20" s="61"/>
       <c r="F20" s="61">
         <f>MAX(MAX(C17:I17),MAX(K17:M17)-N20)+D20</f>
-        <v>10661.450006387617</v>
+        <v>0</v>
       </c>
       <c r="G20" s="61"/>
       <c r="H20" s="61"/>
@@ -3582,7 +3488,7 @@
       <c r="M20" s="61"/>
       <c r="N20" s="61">
         <f>O17</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O20" s="61"/>
       <c r="P20" s="61"/>
@@ -3591,12 +3497,12 @@
       <c r="S20" s="70"/>
       <c r="T20" s="61">
         <f>IF(V$8+X$8+Y$8+W$8+AD$8+AF$8+AG$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="U20" s="61"/>
       <c r="V20" s="61">
         <f>MAX(MAX(S17:Y17),MAX(AA17:AC17)-AD20)+T20</f>
-        <v>10500</v>
+        <v>0</v>
       </c>
       <c r="W20" s="61"/>
       <c r="X20" s="61"/>
@@ -3610,20 +3516,20 @@
       <c r="AG20" s="73"/>
       <c r="AH20" s="8"/>
     </row>
-    <row r="21" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="134" t="s">
+    <row r="21" spans="1:42" s="68" customFormat="1" hidden="1">
+      <c r="A21" s="99" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="134"/>
+      <c r="B21" s="99"/>
       <c r="C21" s="70"/>
       <c r="D21" s="61">
         <f>IF(F$8+H$8+I$8+N$8+P$8+Q$8+O$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E21" s="61"/>
       <c r="F21" s="61">
         <f>G17</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G21" s="61"/>
       <c r="H21" s="61"/>
@@ -3634,7 +3540,7 @@
       <c r="M21" s="61"/>
       <c r="N21" s="61">
         <f>MAX(MAX(K17:Q17),MAX(C17:E17)-F21)+D21</f>
-        <v>10761.450006387617</v>
+        <v>0</v>
       </c>
       <c r="O21" s="61"/>
       <c r="P21" s="61"/>
@@ -3643,12 +3549,12 @@
       <c r="S21" s="70"/>
       <c r="T21" s="61">
         <f>IF(V$8+X$8+Y$8+AD$8+AF$8+AG$8+AE$8=0,0,10000)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="U21" s="61"/>
       <c r="V21" s="61">
         <f>W17</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W21" s="61"/>
       <c r="X21" s="61"/>
@@ -3657,12 +3563,12 @@
       <c r="AA21" s="72"/>
       <c r="AD21" s="68">
         <f>MAX(MAX(AA17:AG17),MAX(S17:U17)-V21)+T21</f>
-        <v>10500</v>
+        <v>0</v>
       </c>
       <c r="AG21" s="73"/>
       <c r="AH21" s="8"/>
     </row>
-    <row r="22" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:42" s="68" customFormat="1" hidden="1">
       <c r="A22" s="61"/>
       <c r="B22" s="61"/>
       <c r="C22" s="70"/>
@@ -3693,7 +3599,7 @@
       <c r="AG22" s="73"/>
       <c r="AH22" s="8"/>
     </row>
-    <row r="23" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:42" s="68" customFormat="1" hidden="1">
       <c r="A23" s="61"/>
       <c r="B23" s="61"/>
       <c r="C23" s="70"/>
@@ -3724,7 +3630,7 @@
       <c r="AG23" s="73"/>
       <c r="AH23" s="8"/>
     </row>
-    <row r="24" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:42" s="68" customFormat="1" hidden="1">
       <c r="A24" s="61"/>
       <c r="B24" s="61"/>
       <c r="C24" s="70"/>
@@ -3755,7 +3661,7 @@
       <c r="AG24" s="73"/>
       <c r="AH24" s="8"/>
     </row>
-    <row r="25" spans="1:42" s="68" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:42" s="68" customFormat="1" hidden="1">
       <c r="A25" s="61"/>
       <c r="B25" s="61"/>
       <c r="C25" s="70"/>
@@ -3786,7 +3692,7 @@
       <c r="AG25" s="73"/>
       <c r="AH25" s="8"/>
     </row>
-    <row r="26" spans="1:42" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:42" ht="15" hidden="1" customHeight="1">
       <c r="A26" s="7" t="s">
         <v>43</v>
       </c>
@@ -3824,7 +3730,7 @@
       <c r="AE26" s="77"/>
       <c r="AG26" s="60"/>
     </row>
-    <row r="27" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:42" hidden="1">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="57"/>
@@ -3853,7 +3759,7 @@
       <c r="AA27" s="59"/>
       <c r="AG27" s="60"/>
     </row>
-    <row r="28" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:42" hidden="1">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="57"/>
@@ -3882,94 +3788,94 @@
       <c r="AA28" s="59"/>
       <c r="AG28" s="60"/>
     </row>
-    <row r="29" spans="1:42" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:42" ht="15" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
-      <c r="C29" s="135" t="str">
+      <c r="C29" s="100" t="str">
         <f>C2</f>
-        <v>צפון   -   לוי אשכול</v>
-      </c>
-      <c r="D29" s="136"/>
-      <c r="E29" s="136"/>
-      <c r="F29" s="136"/>
-      <c r="G29" s="136"/>
-      <c r="H29" s="136"/>
-      <c r="I29" s="137"/>
+        <v>צפון</v>
+      </c>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
+      <c r="F29" s="101"/>
+      <c r="G29" s="101"/>
+      <c r="H29" s="101"/>
+      <c r="I29" s="102"/>
       <c r="J29" s="7"/>
-      <c r="K29" s="101" t="str">
+      <c r="K29" s="117" t="str">
         <f>G2</f>
-        <v>דרום   -   לוי אשכול</v>
-      </c>
-      <c r="L29" s="102"/>
-      <c r="M29" s="102"/>
-      <c r="N29" s="102"/>
-      <c r="O29" s="102"/>
-      <c r="P29" s="102"/>
-      <c r="Q29" s="103"/>
+        <v>דרום</v>
+      </c>
+      <c r="L29" s="118"/>
+      <c r="M29" s="118"/>
+      <c r="N29" s="118"/>
+      <c r="O29" s="118"/>
+      <c r="P29" s="118"/>
+      <c r="Q29" s="119"/>
       <c r="R29" s="7"/>
-      <c r="S29" s="107" t="str">
+      <c r="S29" s="123" t="str">
         <f>K2</f>
-        <v>מזרח   -   יהודה הלוי</v>
-      </c>
-      <c r="T29" s="108"/>
-      <c r="U29" s="108"/>
-      <c r="V29" s="108"/>
-      <c r="W29" s="108"/>
-      <c r="X29" s="108"/>
-      <c r="Y29" s="109"/>
-      <c r="AA29" s="113" t="str">
+        <v>מזרח</v>
+      </c>
+      <c r="T29" s="124"/>
+      <c r="U29" s="124"/>
+      <c r="V29" s="124"/>
+      <c r="W29" s="124"/>
+      <c r="X29" s="124"/>
+      <c r="Y29" s="125"/>
+      <c r="AA29" s="129" t="str">
         <f>O2</f>
-        <v>מערב   -   מיכאל וולך</v>
-      </c>
-      <c r="AB29" s="114"/>
-      <c r="AC29" s="114"/>
-      <c r="AD29" s="114"/>
-      <c r="AE29" s="114"/>
-      <c r="AF29" s="114"/>
-      <c r="AG29" s="115"/>
-    </row>
-    <row r="30" spans="1:42" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>מערב</v>
+      </c>
+      <c r="AB29" s="130"/>
+      <c r="AC29" s="130"/>
+      <c r="AD29" s="130"/>
+      <c r="AE29" s="130"/>
+      <c r="AF29" s="130"/>
+      <c r="AG29" s="131"/>
+    </row>
+    <row r="30" spans="1:42" ht="15" customHeight="1" thickBot="1">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
-      <c r="C30" s="138"/>
-      <c r="D30" s="139"/>
-      <c r="E30" s="139"/>
-      <c r="F30" s="139"/>
-      <c r="G30" s="139"/>
-      <c r="H30" s="139"/>
-      <c r="I30" s="140"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="104"/>
+      <c r="E30" s="104"/>
+      <c r="F30" s="104"/>
+      <c r="G30" s="104"/>
+      <c r="H30" s="104"/>
+      <c r="I30" s="105"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="104"/>
-      <c r="L30" s="105"/>
-      <c r="M30" s="105"/>
-      <c r="N30" s="105"/>
-      <c r="O30" s="105"/>
-      <c r="P30" s="105"/>
-      <c r="Q30" s="106"/>
+      <c r="K30" s="120"/>
+      <c r="L30" s="121"/>
+      <c r="M30" s="121"/>
+      <c r="N30" s="121"/>
+      <c r="O30" s="121"/>
+      <c r="P30" s="121"/>
+      <c r="Q30" s="122"/>
       <c r="R30" s="7"/>
-      <c r="S30" s="110"/>
-      <c r="T30" s="111"/>
-      <c r="U30" s="111"/>
-      <c r="V30" s="111"/>
-      <c r="W30" s="111"/>
-      <c r="X30" s="111"/>
-      <c r="Y30" s="112"/>
-      <c r="AA30" s="116"/>
-      <c r="AB30" s="117"/>
-      <c r="AC30" s="117"/>
-      <c r="AD30" s="117"/>
-      <c r="AE30" s="117"/>
-      <c r="AF30" s="117"/>
-      <c r="AG30" s="118"/>
-    </row>
-    <row r="31" spans="1:42" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:42" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S30" s="126"/>
+      <c r="T30" s="127"/>
+      <c r="U30" s="127"/>
+      <c r="V30" s="127"/>
+      <c r="W30" s="127"/>
+      <c r="X30" s="127"/>
+      <c r="Y30" s="128"/>
+      <c r="AA30" s="132"/>
+      <c r="AB30" s="133"/>
+      <c r="AC30" s="133"/>
+      <c r="AD30" s="133"/>
+      <c r="AE30" s="133"/>
+      <c r="AF30" s="133"/>
+      <c r="AG30" s="134"/>
+    </row>
+    <row r="31" spans="1:42" ht="15" customHeight="1"/>
+    <row r="32" spans="1:42" ht="15" customHeight="1">
       <c r="N32" s="9"/>
     </row>
-    <row r="33" spans="3:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:28" ht="15.75" customHeight="1">
       <c r="N33" s="9"/>
     </row>
-    <row r="34" spans="3:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="3:28" ht="15" customHeight="1" thickBot="1">
       <c r="O34" s="7"/>
       <c r="P34" s="7"/>
       <c r="Q34" s="7"/>
@@ -3985,46 +3891,44 @@
       <c r="AA34" s="7"/>
       <c r="AB34" s="7"/>
     </row>
-    <row r="35" spans="3:28" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H35" s="141" t="str">
+    <row r="35" spans="3:28" ht="15" customHeight="1" thickBot="1">
+      <c r="H35" s="106" t="str">
         <f>AP19</f>
         <v>תקין</v>
       </c>
-      <c r="I35" s="142"/>
-      <c r="J35" s="142"/>
-      <c r="K35" s="142"/>
-      <c r="L35" s="143"/>
+      <c r="I35" s="107"/>
+      <c r="J35" s="107"/>
+      <c r="K35" s="107"/>
+      <c r="L35" s="108"/>
       <c r="O35" s="7"/>
-      <c r="R35" s="99" t="s">
+      <c r="R35" s="115" t="s">
         <v>44</v>
       </c>
-      <c r="S35" s="100"/>
+      <c r="S35" s="116"/>
       <c r="U35" s="7"/>
-      <c r="V35" s="99" t="s">
+      <c r="V35" s="115" t="s">
         <v>45</v>
       </c>
-      <c r="W35" s="100"/>
+      <c r="W35" s="116"/>
       <c r="X35" s="78"/>
       <c r="Y35" s="78"/>
-      <c r="Z35" s="99" t="s">
+      <c r="Z35" s="115" t="s">
         <v>46</v>
       </c>
-      <c r="AA35" s="100"/>
+      <c r="AA35" s="116"/>
       <c r="AB35" s="7"/>
     </row>
-    <row r="36" spans="3:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H36" s="144"/>
-      <c r="I36" s="145"/>
-      <c r="J36" s="145"/>
-      <c r="K36" s="145"/>
-      <c r="L36" s="146"/>
+    <row r="36" spans="3:28" ht="15.75" customHeight="1" thickBot="1">
+      <c r="H36" s="109"/>
+      <c r="I36" s="110"/>
+      <c r="J36" s="110"/>
+      <c r="K36" s="110"/>
+      <c r="L36" s="111"/>
       <c r="O36" s="7"/>
       <c r="R36" s="94" t="s">
         <v>47</v>
       </c>
-      <c r="S36" s="98" t="s">
-        <v>70</v>
-      </c>
+      <c r="S36" s="98"/>
       <c r="U36" s="7"/>
       <c r="V36" s="79">
         <v>1800</v>
@@ -4035,29 +3939,27 @@
       <c r="X36" s="78"/>
       <c r="Y36" s="78"/>
       <c r="Z36" s="81">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA36" s="82" t="s">
         <v>49</v>
       </c>
       <c r="AB36" s="7"/>
     </row>
-    <row r="37" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H37" s="144"/>
-      <c r="I37" s="145"/>
-      <c r="J37" s="145"/>
-      <c r="K37" s="145"/>
-      <c r="L37" s="146"/>
+    <row r="37" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
+      <c r="H37" s="109"/>
+      <c r="I37" s="110"/>
+      <c r="J37" s="110"/>
+      <c r="K37" s="110"/>
+      <c r="L37" s="111"/>
       <c r="O37" s="7"/>
       <c r="R37" s="94" t="s">
         <v>50</v>
       </c>
-      <c r="S37" s="96">
-        <v>2799.01</v>
-      </c>
+      <c r="S37" s="96"/>
       <c r="U37" s="7"/>
       <c r="V37" s="83">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W37" s="84" t="s">
         <v>51</v>
@@ -4072,12 +3974,12 @@
       </c>
       <c r="AB37" s="7"/>
     </row>
-    <row r="38" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H38" s="147"/>
-      <c r="I38" s="148"/>
-      <c r="J38" s="148"/>
-      <c r="K38" s="148"/>
-      <c r="L38" s="149"/>
+    <row r="38" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
+      <c r="H38" s="112"/>
+      <c r="I38" s="113"/>
+      <c r="J38" s="113"/>
+      <c r="K38" s="113"/>
+      <c r="L38" s="114"/>
       <c r="O38" s="7"/>
       <c r="R38" s="94" t="s">
         <v>53</v>
@@ -4085,7 +3987,7 @@
       <c r="S38" s="96"/>
       <c r="U38" s="7"/>
       <c r="V38" s="83">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W38" s="84" t="s">
         <v>54</v>
@@ -4100,7 +4002,7 @@
       </c>
       <c r="AB38" s="7"/>
     </row>
-    <row r="39" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
@@ -4119,9 +4021,7 @@
       <c r="R39" s="94" t="s">
         <v>56</v>
       </c>
-      <c r="S39" s="96">
-        <v>1</v>
-      </c>
+      <c r="S39" s="96"/>
       <c r="T39" s="7"/>
       <c r="U39" s="7"/>
       <c r="V39" s="83">
@@ -4140,7 +4040,7 @@
       </c>
       <c r="AB39" s="7"/>
     </row>
-    <row r="40" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
@@ -4178,7 +4078,7 @@
       </c>
       <c r="AB40" s="7"/>
     </row>
-    <row r="41" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="O41" s="7"/>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
@@ -4202,7 +4102,7 @@
       </c>
       <c r="AB41" s="7"/>
     </row>
-    <row r="42" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
       <c r="Q42" s="7"/>
@@ -4222,7 +4122,7 @@
       <c r="AA42" s="78"/>
       <c r="AB42" s="7"/>
     </row>
-    <row r="43" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="O43" s="7"/>
       <c r="P43" s="7"/>
       <c r="Q43" s="7"/>
@@ -4242,7 +4142,7 @@
       <c r="AA43" s="78"/>
       <c r="AB43" s="7"/>
     </row>
-    <row r="44" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
       <c r="Q44" s="7"/>
@@ -4251,7 +4151,7 @@
       <c r="T44" s="7"/>
       <c r="U44" s="7"/>
       <c r="V44" s="83">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W44" s="84" t="s">
         <v>66</v>
@@ -4262,7 +4162,7 @@
       <c r="AA44" s="78"/>
       <c r="AB44" s="7"/>
     </row>
-    <row r="45" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="3:28" ht="16.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="O45" s="7"/>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
@@ -4282,7 +4182,7 @@
       <c r="AA45" s="78"/>
       <c r="AB45" s="7"/>
     </row>
-    <row r="46" spans="3:28" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="3:28" ht="15" customHeight="1" thickTop="1" thickBot="1">
       <c r="V46" s="92">
         <v>1</v>
       </c>
@@ -4296,11 +4196,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C29:I30"/>
-    <mergeCell ref="H35:L38"/>
-    <mergeCell ref="V35:W35"/>
     <mergeCell ref="Z35:AA35"/>
     <mergeCell ref="K29:Q30"/>
     <mergeCell ref="S29:Y30"/>
@@ -4311,35 +4206,35 @@
     <mergeCell ref="O2:R2"/>
     <mergeCell ref="V2:Y2"/>
     <mergeCell ref="R35:S35"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C29:I30"/>
+    <mergeCell ref="H35:L38"/>
+    <mergeCell ref="V35:W35"/>
   </mergeCells>
+  <conditionalFormatting sqref="C8:Q9">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H35:L38">
-    <cfRule type="containsText" dxfId="6" priority="13" operator="containsText" text="תקין">
+    <cfRule type="containsText" dxfId="4" priority="13" operator="containsText" text="תקין">
       <formula>NOT(ISERROR(SEARCH("תקין",H35)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7 J10:J31">
-    <cfRule type="cellIs" dxfId="5" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S8:Y9">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z40:Z41">
-    <cfRule type="cellIs" dxfId="4" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="greaterThan">
       <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8:J9">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K8:Q9">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S8:Y9">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA8:AG9">
@@ -4404,17 +4299,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="N34:P37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="34" spans="14:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="35" spans="14:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="14:16" ht="15" customHeight="1" thickBot="1"/>
+    <row r="35" spans="14:16">
       <c r="N35" s="150" t="s">
         <v>69</v>
       </c>
       <c r="O35" s="151"/>
       <c r="P35" s="152"/>
     </row>
-    <row r="36" spans="14:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="14:16">
       <c r="N36" s="2">
         <v>4</v>
       </c>
@@ -4425,7 +4320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="14:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="14:16" ht="15" customHeight="1" thickBot="1">
       <c r="N37" s="4">
         <v>1400</v>
       </c>
@@ -4448,7 +4343,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>